<commit_message>
FIX: missing column on PIA model, and updated template
</commit_message>
<xml_diff>
--- a/templates/PIA_Modelo de datos_template.xlsx
+++ b/templates/PIA_Modelo de datos_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspaces\OCR_tests - uv\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F5D0773-0AE8-4549-9DA2-5D5F6E15A905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB9CF5E5-4EE3-49AD-8E4F-93CF22A5EB45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2BC6707C-099C-46BC-8C2F-C7B9585D3BFF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>Nombre del Archivo</t>
   </si>
@@ -59,9 +59,6 @@
     <t>Descripción de la finalidad y objetivos a alcanzar al realizar un PIA</t>
   </si>
   <si>
-    <t>1.1.2. Análisis de la necesidad del PIA - Situaciones que aconsejan realizar una mnueva evaluación de impacto o actualizar la ya realizada para este tratamiento de datos</t>
-  </si>
-  <si>
     <t>¿Se encuentra la presente actividad de tratamiento en los supuestos indicados como de "Riesgo alto" para los derechos y libertades de las personas o existen otros motivos que justifiquen elaborar un PIA</t>
   </si>
   <si>
@@ -198,6 +195,12 @@
   </si>
   <si>
     <t>3.10. Seguridad de los tratamientos</t>
+  </si>
+  <si>
+    <t>1.1.2. Análisis de la necesidad del PIA - Situaciones que aconsejan realizar una nueva evaluación de impacto o actualizar la ya realizada para este tratamiento de datos</t>
+  </si>
+  <si>
+    <t>2.1.7 Comprensión de la evaluación - Descripción detallada del programa, proceso o sistema a evaluar</t>
   </si>
 </sst>
 </file>
@@ -599,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E69E6B67-23EC-4E98-86B0-B4DAF1BFB0EF}">
-  <dimension ref="A1:BB3"/>
+  <dimension ref="A1:BC3"/>
   <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.296875" style="1" bestFit="1" customWidth="1"/>
@@ -645,21 +648,22 @@
     <col min="41" max="41" width="24.59765625" style="1" bestFit="1" customWidth="1"/>
     <col min="42" max="42" width="53.69921875" style="1" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="65.09765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="21.8984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="47.796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="24" style="1" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="32.59765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="25" style="1" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="31" style="1" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="29.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="32.19921875" style="1" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="25.09765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="24.8984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="54" max="55" width="29.09765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="56" max="16384" width="8.69921875" style="1"/>
+    <col min="44" max="44" width="65.09765625" style="1" customWidth="1"/>
+    <col min="45" max="45" width="21.8984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="47.796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="24" style="1" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="32.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="25" style="1" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="31" style="1" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="29.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="32.19921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="25.09765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="24.8984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="55" max="56" width="29.09765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="57" max="16384" width="8.69921875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:55" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -682,152 +686,155 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AK1" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AL1" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AM1" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AN1" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AO1" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AP1" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AQ1" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AR1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AS1" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AT1" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AU1" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AV1" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AW1" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AX1" t="s">
         <v>47</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AY1" t="s">
         <v>48</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AZ1" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="BA1" t="s">
         <v>50</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BB1" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BC1" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" t="s">
-        <v>53</v>
-      </c>
     </row>
-    <row r="2" spans="1:54" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:55" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="1:54" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:55" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>